<commit_message>
Change winning criteria from 5 to 3 correct answers
</commit_message>
<xml_diff>
--- a/Raw data.xlsx
+++ b/Raw data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thanakritpan\Desktop\ด่วนๆ\SeminarWebGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3B992E2-932F-497D-BA67-E64BA7B274D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34706BE2-621B-47A5-BA59-E50B747FD248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{736536AE-1CCD-4821-9CDB-3622C732E062}"/>
   </bookViews>
@@ -487,7 +487,7 @@
         <v>5</v>
       </c>
       <c r="D3">
-        <v>93</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>